<commit_message>
Adjust for new endpoint
Signed-off-by: Walter Nascimento <walter.nascimento.barroso@gmail.com>
</commit_message>
<xml_diff>
--- a/src/reports/mapa_km/template.xlsx
+++ b/src/reports/mapa_km/template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t xml:space="preserve">Mapa por deslocação em viatura própria </t>
   </si>
@@ -24,16 +24,10 @@
     <t>Empresa:</t>
   </si>
   <si>
-    <t>FULGORABSTRACTO - LDA</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
     <t xml:space="preserve">Morada: </t>
-  </si>
-  <si>
-    <t>Rua Caseta, Nº 9, 1º Esq. Trás</t>
   </si>
   <si>
     <t>Mês:</t>
@@ -43,9 +37,6 @@
   </si>
   <si>
     <t xml:space="preserve">Nº de Contribuinte: </t>
-  </si>
-  <si>
-    <t>Fevereiro</t>
   </si>
   <si>
     <t>Dia</t>
@@ -63,15 +54,6 @@
     <t>Nº de KMS</t>
   </si>
   <si>
-    <t>Deslocação para execução de tarefas</t>
-  </si>
-  <si>
-    <t>Lisboa</t>
-  </si>
-  <si>
-    <t>Braga</t>
-  </si>
-  <si>
     <t>Total de KMS:</t>
   </si>
   <si>
@@ -87,16 +69,10 @@
     <t>Nome:</t>
   </si>
   <si>
-    <t>Walter Nascimento Barroso</t>
-  </si>
-  <si>
     <t>Nº Fiscal:</t>
   </si>
   <si>
     <t>Viatura:</t>
-  </si>
-  <si>
-    <t>85-58-XA</t>
   </si>
   <si>
     <t xml:space="preserve">Data: </t>
@@ -209,7 +185,7 @@
       <name val="Arial Narrow"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -230,24 +206,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF6B26B"/>
-        <bgColor rgb="FFF6B26B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor theme="0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="13">
     <border/>
     <border>
       <left style="thin">
@@ -336,32 +300,12 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="hair">
         <color rgb="FF000000"/>
       </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
     </border>
     <border>
       <left style="thin">
@@ -395,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="47">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -430,7 +374,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,7 +386,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -450,12 +394,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="12" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="10" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="9" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf borderId="6" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
@@ -464,26 +402,23 @@
     </xf>
     <xf borderId="6" fillId="0" fontId="12" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="12" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="13" fillId="6" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="13" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="12" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="11" fillId="4" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="11" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="13" fillId="6" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="11" fillId="4" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="14" fillId="2" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="12" fillId="2" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="12" fillId="2" fontId="4" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="10" fillId="2" fontId="4" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
@@ -506,7 +441,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="5" fillId="2" fontId="9" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
@@ -787,67 +722,59 @@
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>2</v>
-      </c>
+      <c r="A4" s="4"/>
       <c r="B4" s="5"/>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
       <c r="A5" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B5" s="9"/>
       <c r="C5" s="6"/>
       <c r="D5" s="10" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
       <c r="A6" s="8"/>
       <c r="B6" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="14">
-        <v>5.18688003E8</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C6" s="14"/>
       <c r="D6" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>9</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E6" s="15"/>
       <c r="F6" s="16">
         <v>2026.0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>10</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>13</v>
       </c>
       <c r="E8" s="19"/>
       <c r="F8" s="17" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
@@ -861,23 +788,17 @@
       <c r="F9" s="23"/>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="24">
+      <c r="A10" s="20">
         <v>2.0</v>
       </c>
-      <c r="B10" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>16</v>
-      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="22"/>
       <c r="E10" s="6"/>
-      <c r="F10" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F10" s="23"/>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="24">
+      <c r="A11" s="20">
         <v>3.0</v>
       </c>
       <c r="B11" s="21"/>
@@ -887,7 +808,7 @@
       <c r="F11" s="23"/>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="24">
+      <c r="A12" s="20">
         <v>4.0</v>
       </c>
       <c r="B12" s="21"/>
@@ -897,7 +818,7 @@
       <c r="F12" s="23"/>
     </row>
     <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="24">
+      <c r="A13" s="20">
         <v>5.0</v>
       </c>
       <c r="B13" s="21"/>
@@ -907,20 +828,14 @@
       <c r="F13" s="23"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="24">
+      <c r="A14" s="20">
         <v>6.0</v>
       </c>
-      <c r="B14" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>17</v>
-      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="22"/>
       <c r="E14" s="6"/>
-      <c r="F14" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F14" s="23"/>
     </row>
     <row r="15" ht="21.75" customHeight="1">
       <c r="A15" s="20">
@@ -943,23 +858,17 @@
       <c r="F16" s="23"/>
     </row>
     <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="24">
+      <c r="A17" s="20">
         <v>9.0</v>
       </c>
-      <c r="B17" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>16</v>
-      </c>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="22"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F17" s="23"/>
     </row>
     <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="24">
+      <c r="A18" s="20">
         <v>10.0</v>
       </c>
       <c r="B18" s="21"/>
@@ -969,23 +878,17 @@
       <c r="F18" s="23"/>
     </row>
     <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="24">
+      <c r="A19" s="20">
         <v>11.0</v>
       </c>
-      <c r="B19" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>17</v>
-      </c>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
       <c r="D19" s="22"/>
       <c r="E19" s="6"/>
-      <c r="F19" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F19" s="23"/>
     </row>
     <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="24">
+      <c r="A20" s="20">
         <v>12.0</v>
       </c>
       <c r="B20" s="21"/>
@@ -995,7 +898,7 @@
       <c r="F20" s="23"/>
     </row>
     <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="24">
+      <c r="A21" s="20">
         <v>13.0</v>
       </c>
       <c r="B21" s="21"/>
@@ -1025,7 +928,7 @@
       <c r="F23" s="23"/>
     </row>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="24">
+      <c r="A24" s="20">
         <v>16.0</v>
       </c>
       <c r="B24" s="21"/>
@@ -1035,7 +938,7 @@
       <c r="F24" s="23"/>
     </row>
     <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="25">
+      <c r="A25" s="20">
         <v>17.0</v>
       </c>
       <c r="B25" s="21"/>
@@ -1045,23 +948,17 @@
       <c r="F25" s="23"/>
     </row>
     <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="24">
+      <c r="A26" s="20">
         <v>18.0</v>
       </c>
-      <c r="B26" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>16</v>
-      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="22"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F26" s="23"/>
     </row>
     <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="24">
+      <c r="A27" s="20">
         <v>19.0</v>
       </c>
       <c r="B27" s="21"/>
@@ -1071,20 +968,14 @@
       <c r="F27" s="23"/>
     </row>
     <row r="28" ht="21.75" customHeight="1">
-      <c r="A28" s="24">
+      <c r="A28" s="20">
         <v>20.0</v>
       </c>
-      <c r="B28" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>17</v>
-      </c>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="22"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F28" s="23"/>
     </row>
     <row r="29" ht="21.75" customHeight="1">
       <c r="A29" s="20">
@@ -1107,7 +998,7 @@
       <c r="F30" s="23"/>
     </row>
     <row r="31" ht="21.75" customHeight="1">
-      <c r="A31" s="24">
+      <c r="A31" s="20">
         <v>23.0</v>
       </c>
       <c r="B31" s="21"/>
@@ -1117,33 +1008,27 @@
       <c r="F31" s="23"/>
     </row>
     <row r="32" ht="21.75" customHeight="1">
-      <c r="A32" s="24">
+      <c r="A32" s="20">
         <v>24.0</v>
       </c>
       <c r="B32" s="21"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="27"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="25"/>
       <c r="E32" s="6"/>
-      <c r="F32" s="28"/>
+      <c r="F32" s="26"/>
     </row>
     <row r="33" ht="21.75" customHeight="1">
-      <c r="A33" s="24">
+      <c r="A33" s="20">
         <v>25.0</v>
       </c>
-      <c r="B33" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>16</v>
-      </c>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
       <c r="D33" s="22"/>
       <c r="E33" s="6"/>
-      <c r="F33" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F33" s="23"/>
     </row>
     <row r="34" ht="21.75" customHeight="1">
-      <c r="A34" s="24">
+      <c r="A34" s="20">
         <v>26.0</v>
       </c>
       <c r="B34" s="21"/>
@@ -1153,20 +1038,14 @@
       <c r="F34" s="23"/>
     </row>
     <row r="35" ht="21.75" customHeight="1">
-      <c r="A35" s="24">
+      <c r="A35" s="20">
         <v>27.0</v>
       </c>
-      <c r="B35" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>17</v>
-      </c>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
       <c r="D35" s="22"/>
       <c r="E35" s="6"/>
-      <c r="F35" s="23">
-        <v>363.0</v>
-      </c>
+      <c r="F35" s="23"/>
     </row>
     <row r="36" ht="21.75" customHeight="1">
       <c r="A36" s="20">
@@ -1179,7 +1058,9 @@
       <c r="F36" s="23"/>
     </row>
     <row r="37" ht="21.75" customHeight="1">
-      <c r="A37" s="24"/>
+      <c r="A37" s="20">
+        <v>29.0</v>
+      </c>
       <c r="B37" s="21"/>
       <c r="C37" s="21"/>
       <c r="D37" s="22"/>
@@ -1187,15 +1068,19 @@
       <c r="F37" s="23"/>
     </row>
     <row r="38" ht="21.75" customHeight="1">
-      <c r="A38" s="29"/>
+      <c r="A38" s="20">
+        <v>30.0</v>
+      </c>
       <c r="B38" s="21"/>
       <c r="C38" s="21"/>
-      <c r="D38" s="27"/>
+      <c r="D38" s="25"/>
       <c r="E38" s="6"/>
       <c r="F38" s="23"/>
     </row>
     <row r="39" ht="21.75" customHeight="1">
-      <c r="A39" s="16"/>
+      <c r="A39" s="20">
+        <v>31.0</v>
+      </c>
       <c r="B39" s="21"/>
       <c r="C39" s="21"/>
       <c r="D39" s="22"/>
@@ -1203,94 +1088,84 @@
       <c r="F39" s="23"/>
     </row>
     <row r="40" ht="21.75" customHeight="1">
-      <c r="A40" s="30"/>
-      <c r="E40" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="F40" s="32">
+      <c r="A40" s="27"/>
+      <c r="E40" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40" s="29">
         <f>SUM(F9:F39)</f>
-        <v>2904</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" ht="21.75" customHeight="1">
-      <c r="E41" s="31"/>
+      <c r="E41" s="28"/>
     </row>
     <row r="42" ht="24.75" customHeight="1">
-      <c r="A42" s="33"/>
-      <c r="B42" s="34"/>
-      <c r="C42" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="D42" s="36">
+      <c r="A42" s="30"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" s="33">
         <v>0.4</v>
       </c>
-      <c r="E42" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="F42" s="37">
+      <c r="E42" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="34">
         <f>F40*D42</f>
-        <v>1161.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="38"/>
-      <c r="C43" s="38"/>
-      <c r="D43" s="38"/>
-      <c r="F43" s="31"/>
+      <c r="B43" s="35"/>
+      <c r="C43" s="35"/>
+      <c r="D43" s="35"/>
+      <c r="F43" s="28"/>
     </row>
     <row r="44" ht="19.5" customHeight="1">
       <c r="A44" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45" ht="19.5" customHeight="1">
       <c r="A45" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B45" s="39" t="s">
-        <v>23</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B45" s="36"/>
       <c r="C45" s="6"/>
-      <c r="D45" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="E45" s="41">
-        <v>3.15929529E8</v>
-      </c>
-      <c r="F45" s="42"/>
+      <c r="D45" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="E45" s="38"/>
+      <c r="F45" s="39"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
       <c r="A46" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B46" s="39" t="s">
-        <v>5</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B46" s="36"/>
       <c r="C46" s="6"/>
-      <c r="D46" s="43" t="s">
-        <v>25</v>
-      </c>
-      <c r="E46" s="44" t="s">
-        <v>26</v>
-      </c>
-      <c r="F46" s="42"/>
+      <c r="D46" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="E46" s="41"/>
+      <c r="F46" s="39"/>
     </row>
     <row r="47" ht="19.5" customHeight="1">
       <c r="A47" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B47" s="45">
-        <v>46081.0</v>
-      </c>
-      <c r="C47" s="46" t="s">
-        <v>28</v>
-      </c>
-      <c r="D47" s="47" t="s">
-        <v>29</v>
-      </c>
-      <c r="E47" s="48"/>
-      <c r="F47" s="49" t="s">
-        <v>3</v>
+        <v>19</v>
+      </c>
+      <c r="B47" s="42"/>
+      <c r="C47" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="D47" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="E47" s="45"/>
+      <c r="F47" s="46" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1"/>
@@ -2252,15 +2127,15 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D10:E10"/>
     <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
     <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D17:E17"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="D21:E21"/>
@@ -2269,20 +2144,20 @@
     <mergeCell ref="D24:E24"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
     <mergeCell ref="D36:E36"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="B46:C46"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
     <mergeCell ref="D33:E33"/>
   </mergeCells>
   <printOptions/>

</xml_diff>